<commit_message>
fix: stop asking anyone to type the workbook anchor date
Vincent entered the Thursday and the sheet showed Monday. Not a display
fault: the cell really held a Monday (6 July instead of 6 August). Typing a
date on a phone depends on system language and day/month order, and nothing
in the sheet said the value was wrong.

The anchor is now =TODAY(), so the normal case needs no typing at all. It
stays editable for a late fill, with the weekday spelled out next to it
(dddd format, not TEXT() whose language varies) and a WEEKDAY(...,2)=4 check.
The covered period is echoed at the top of the Passages sheet, where it is
actually read.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SAGB14yDJZ1V2SSANXBgTH
</commit_message>
<xml_diff>
--- a/docs/modele-passages.xlsx
+++ b/docs/modele-passages.xlsx
@@ -86,15 +86,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -482,641 +483,653 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Commence par indiquer la date d'envoi dans la feuille « Periode ».</t>
-        </is>
+          <t>Dates proposées, de :</t>
+        </is>
+      </c>
+      <c r="B2" s="2">
+        <f>MIN(Periode!$B$7:$B$27)</f>
+        <v/>
+      </c>
+      <c r="C2" s="2">
+        <f>MAX(Periode!$B$7:$B$27)</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>Periode!$D$1</f>
+        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>date_visite</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>magasin</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>commercial</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>heure_arrivee</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>heure_depart</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
+      <c r="A5" s="2" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
+      <c r="A6" s="2" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
+      <c r="A7" s="2" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
+      <c r="A8" s="2" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
+      <c r="A9" s="2" t="n"/>
       <c r="D9" s="5" t="n"/>
       <c r="E9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
+      <c r="A10" s="2" t="n"/>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
+      <c r="A11" s="2" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
+      <c r="A12" s="2" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
+      <c r="A13" s="2" t="n"/>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
+      <c r="A14" s="2" t="n"/>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
+      <c r="A15" s="2" t="n"/>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
+      <c r="A16" s="2" t="n"/>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n"/>
+      <c r="A17" s="2" t="n"/>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n"/>
+      <c r="A18" s="2" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n"/>
+      <c r="A19" s="2" t="n"/>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n"/>
+      <c r="A20" s="2" t="n"/>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n"/>
+      <c r="A21" s="2" t="n"/>
       <c r="D21" s="5" t="n"/>
       <c r="E21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
+      <c r="A22" s="2" t="n"/>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
+      <c r="A23" s="2" t="n"/>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n"/>
+      <c r="A24" s="2" t="n"/>
       <c r="D24" s="5" t="n"/>
       <c r="E24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
+      <c r="A25" s="2" t="n"/>
       <c r="D25" s="5" t="n"/>
       <c r="E25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n"/>
+      <c r="A26" s="2" t="n"/>
       <c r="D26" s="5" t="n"/>
       <c r="E26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n"/>
+      <c r="A27" s="2" t="n"/>
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n"/>
+      <c r="A28" s="2" t="n"/>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n"/>
+      <c r="A29" s="2" t="n"/>
       <c r="D29" s="5" t="n"/>
       <c r="E29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n"/>
+      <c r="A30" s="2" t="n"/>
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="5" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n"/>
+      <c r="A31" s="2" t="n"/>
       <c r="D31" s="5" t="n"/>
       <c r="E31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n"/>
+      <c r="A32" s="2" t="n"/>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n"/>
+      <c r="A33" s="2" t="n"/>
       <c r="D33" s="5" t="n"/>
       <c r="E33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
+      <c r="A34" s="2" t="n"/>
       <c r="D34" s="5" t="n"/>
       <c r="E34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n"/>
+      <c r="A35" s="2" t="n"/>
       <c r="D35" s="5" t="n"/>
       <c r="E35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n"/>
+      <c r="A36" s="2" t="n"/>
       <c r="D36" s="5" t="n"/>
       <c r="E36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n"/>
+      <c r="A37" s="2" t="n"/>
       <c r="D37" s="5" t="n"/>
       <c r="E37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n"/>
+      <c r="A38" s="2" t="n"/>
       <c r="D38" s="5" t="n"/>
       <c r="E38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n"/>
+      <c r="A39" s="2" t="n"/>
       <c r="D39" s="5" t="n"/>
       <c r="E39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n"/>
+      <c r="A40" s="2" t="n"/>
       <c r="D40" s="5" t="n"/>
       <c r="E40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n"/>
+      <c r="A41" s="2" t="n"/>
       <c r="D41" s="5" t="n"/>
       <c r="E41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n"/>
+      <c r="A42" s="2" t="n"/>
       <c r="D42" s="5" t="n"/>
       <c r="E42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n"/>
+      <c r="A43" s="2" t="n"/>
       <c r="D43" s="5" t="n"/>
       <c r="E43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n"/>
+      <c r="A44" s="2" t="n"/>
       <c r="D44" s="5" t="n"/>
       <c r="E44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n"/>
+      <c r="A45" s="2" t="n"/>
       <c r="D45" s="5" t="n"/>
       <c r="E45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n"/>
+      <c r="A46" s="2" t="n"/>
       <c r="D46" s="5" t="n"/>
       <c r="E46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n"/>
+      <c r="A47" s="2" t="n"/>
       <c r="D47" s="5" t="n"/>
       <c r="E47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n"/>
+      <c r="A48" s="2" t="n"/>
       <c r="D48" s="5" t="n"/>
       <c r="E48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n"/>
+      <c r="A49" s="2" t="n"/>
       <c r="D49" s="5" t="n"/>
       <c r="E49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n"/>
+      <c r="A50" s="2" t="n"/>
       <c r="D50" s="5" t="n"/>
       <c r="E50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n"/>
+      <c r="A51" s="2" t="n"/>
       <c r="D51" s="5" t="n"/>
       <c r="E51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="n"/>
+      <c r="A52" s="2" t="n"/>
       <c r="D52" s="5" t="n"/>
       <c r="E52" s="5" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="n"/>
+      <c r="A53" s="2" t="n"/>
       <c r="D53" s="5" t="n"/>
       <c r="E53" s="5" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="n"/>
+      <c r="A54" s="2" t="n"/>
       <c r="D54" s="5" t="n"/>
       <c r="E54" s="5" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n"/>
+      <c r="A55" s="2" t="n"/>
       <c r="D55" s="5" t="n"/>
       <c r="E55" s="5" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n"/>
+      <c r="A56" s="2" t="n"/>
       <c r="D56" s="5" t="n"/>
       <c r="E56" s="5" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="n"/>
+      <c r="A57" s="2" t="n"/>
       <c r="D57" s="5" t="n"/>
       <c r="E57" s="5" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="n"/>
+      <c r="A58" s="2" t="n"/>
       <c r="D58" s="5" t="n"/>
       <c r="E58" s="5" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="n"/>
+      <c r="A59" s="2" t="n"/>
       <c r="D59" s="5" t="n"/>
       <c r="E59" s="5" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="n"/>
+      <c r="A60" s="2" t="n"/>
       <c r="D60" s="5" t="n"/>
       <c r="E60" s="5" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="n"/>
+      <c r="A61" s="2" t="n"/>
       <c r="D61" s="5" t="n"/>
       <c r="E61" s="5" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="n"/>
+      <c r="A62" s="2" t="n"/>
       <c r="D62" s="5" t="n"/>
       <c r="E62" s="5" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="n"/>
+      <c r="A63" s="2" t="n"/>
       <c r="D63" s="5" t="n"/>
       <c r="E63" s="5" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="n"/>
+      <c r="A64" s="2" t="n"/>
       <c r="D64" s="5" t="n"/>
       <c r="E64" s="5" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="n"/>
+      <c r="A65" s="2" t="n"/>
       <c r="D65" s="5" t="n"/>
       <c r="E65" s="5" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="n"/>
+      <c r="A66" s="2" t="n"/>
       <c r="D66" s="5" t="n"/>
       <c r="E66" s="5" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="n"/>
+      <c r="A67" s="2" t="n"/>
       <c r="D67" s="5" t="n"/>
       <c r="E67" s="5" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="n"/>
+      <c r="A68" s="2" t="n"/>
       <c r="D68" s="5" t="n"/>
       <c r="E68" s="5" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="n"/>
+      <c r="A69" s="2" t="n"/>
       <c r="D69" s="5" t="n"/>
       <c r="E69" s="5" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="4" t="n"/>
+      <c r="A70" s="2" t="n"/>
       <c r="D70" s="5" t="n"/>
       <c r="E70" s="5" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="n"/>
+      <c r="A71" s="2" t="n"/>
       <c r="D71" s="5" t="n"/>
       <c r="E71" s="5" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="n"/>
+      <c r="A72" s="2" t="n"/>
       <c r="D72" s="5" t="n"/>
       <c r="E72" s="5" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="n"/>
+      <c r="A73" s="2" t="n"/>
       <c r="D73" s="5" t="n"/>
       <c r="E73" s="5" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="n"/>
+      <c r="A74" s="2" t="n"/>
       <c r="D74" s="5" t="n"/>
       <c r="E74" s="5" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="n"/>
+      <c r="A75" s="2" t="n"/>
       <c r="D75" s="5" t="n"/>
       <c r="E75" s="5" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="n"/>
+      <c r="A76" s="2" t="n"/>
       <c r="D76" s="5" t="n"/>
       <c r="E76" s="5" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="n"/>
+      <c r="A77" s="2" t="n"/>
       <c r="D77" s="5" t="n"/>
       <c r="E77" s="5" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="n"/>
+      <c r="A78" s="2" t="n"/>
       <c r="D78" s="5" t="n"/>
       <c r="E78" s="5" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="4" t="n"/>
+      <c r="A79" s="2" t="n"/>
       <c r="D79" s="5" t="n"/>
       <c r="E79" s="5" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="n"/>
+      <c r="A80" s="2" t="n"/>
       <c r="D80" s="5" t="n"/>
       <c r="E80" s="5" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="4" t="n"/>
+      <c r="A81" s="2" t="n"/>
       <c r="D81" s="5" t="n"/>
       <c r="E81" s="5" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="n"/>
+      <c r="A82" s="2" t="n"/>
       <c r="D82" s="5" t="n"/>
       <c r="E82" s="5" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="n"/>
+      <c r="A83" s="2" t="n"/>
       <c r="D83" s="5" t="n"/>
       <c r="E83" s="5" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="n"/>
+      <c r="A84" s="2" t="n"/>
       <c r="D84" s="5" t="n"/>
       <c r="E84" s="5" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="n"/>
+      <c r="A85" s="2" t="n"/>
       <c r="D85" s="5" t="n"/>
       <c r="E85" s="5" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="4" t="n"/>
+      <c r="A86" s="2" t="n"/>
       <c r="D86" s="5" t="n"/>
       <c r="E86" s="5" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="n"/>
+      <c r="A87" s="2" t="n"/>
       <c r="D87" s="5" t="n"/>
       <c r="E87" s="5" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="n"/>
+      <c r="A88" s="2" t="n"/>
       <c r="D88" s="5" t="n"/>
       <c r="E88" s="5" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="n"/>
+      <c r="A89" s="2" t="n"/>
       <c r="D89" s="5" t="n"/>
       <c r="E89" s="5" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="n"/>
+      <c r="A90" s="2" t="n"/>
       <c r="D90" s="5" t="n"/>
       <c r="E90" s="5" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="n"/>
+      <c r="A91" s="2" t="n"/>
       <c r="D91" s="5" t="n"/>
       <c r="E91" s="5" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="4" t="n"/>
+      <c r="A92" s="2" t="n"/>
       <c r="D92" s="5" t="n"/>
       <c r="E92" s="5" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="n"/>
+      <c r="A93" s="2" t="n"/>
       <c r="D93" s="5" t="n"/>
       <c r="E93" s="5" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="n"/>
+      <c r="A94" s="2" t="n"/>
       <c r="D94" s="5" t="n"/>
       <c r="E94" s="5" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="n"/>
+      <c r="A95" s="2" t="n"/>
       <c r="D95" s="5" t="n"/>
       <c r="E95" s="5" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="n"/>
+      <c r="A96" s="2" t="n"/>
       <c r="D96" s="5" t="n"/>
       <c r="E96" s="5" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="n"/>
+      <c r="A97" s="2" t="n"/>
       <c r="D97" s="5" t="n"/>
       <c r="E97" s="5" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="n"/>
+      <c r="A98" s="2" t="n"/>
       <c r="D98" s="5" t="n"/>
       <c r="E98" s="5" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="n"/>
+      <c r="A99" s="2" t="n"/>
       <c r="D99" s="5" t="n"/>
       <c r="E99" s="5" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="n"/>
+      <c r="A100" s="2" t="n"/>
       <c r="D100" s="5" t="n"/>
       <c r="E100" s="5" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="4" t="n"/>
+      <c r="A101" s="2" t="n"/>
       <c r="D101" s="5" t="n"/>
       <c r="E101" s="5" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="n"/>
+      <c r="A102" s="2" t="n"/>
       <c r="D102" s="5" t="n"/>
       <c r="E102" s="5" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="n"/>
+      <c r="A103" s="2" t="n"/>
       <c r="D103" s="5" t="n"/>
       <c r="E103" s="5" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="4" t="n"/>
+      <c r="A104" s="2" t="n"/>
       <c r="D104" s="5" t="n"/>
       <c r="E104" s="5" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="4" t="n"/>
+      <c r="A105" s="2" t="n"/>
       <c r="D105" s="5" t="n"/>
       <c r="E105" s="5" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="4" t="n"/>
+      <c r="A106" s="2" t="n"/>
       <c r="D106" s="5" t="n"/>
       <c r="E106" s="5" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="4" t="n"/>
+      <c r="A107" s="2" t="n"/>
       <c r="D107" s="5" t="n"/>
       <c r="E107" s="5" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="4" t="n"/>
+      <c r="A108" s="2" t="n"/>
       <c r="D108" s="5" t="n"/>
       <c r="E108" s="5" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="4" t="n"/>
+      <c r="A109" s="2" t="n"/>
       <c r="D109" s="5" t="n"/>
       <c r="E109" s="5" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="4" t="n"/>
+      <c r="A110" s="2" t="n"/>
       <c r="D110" s="5" t="n"/>
       <c r="E110" s="5" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="4" t="n"/>
+      <c r="A111" s="2" t="n"/>
       <c r="D111" s="5" t="n"/>
       <c r="E111" s="5" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="4" t="n"/>
+      <c r="A112" s="2" t="n"/>
       <c r="D112" s="5" t="n"/>
       <c r="E112" s="5" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="4" t="n"/>
+      <c r="A113" s="2" t="n"/>
       <c r="D113" s="5" t="n"/>
       <c r="E113" s="5" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="4" t="n"/>
+      <c r="A114" s="2" t="n"/>
       <c r="D114" s="5" t="n"/>
       <c r="E114" s="5" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="4" t="n"/>
+      <c r="A115" s="2" t="n"/>
       <c r="D115" s="5" t="n"/>
       <c r="E115" s="5" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="4" t="n"/>
+      <c r="A116" s="2" t="n"/>
       <c r="D116" s="5" t="n"/>
       <c r="E116" s="5" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="4" t="n"/>
+      <c r="A117" s="2" t="n"/>
       <c r="D117" s="5" t="n"/>
       <c r="E117" s="5" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="4" t="n"/>
+      <c r="A118" s="2" t="n"/>
       <c r="D118" s="5" t="n"/>
       <c r="E118" s="5" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="4" t="n"/>
+      <c r="A119" s="2" t="n"/>
       <c r="D119" s="5" t="n"/>
       <c r="E119" s="5" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="4" t="n"/>
+      <c r="A120" s="2" t="n"/>
       <c r="D120" s="5" t="n"/>
       <c r="E120" s="5" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="4" t="n"/>
+      <c r="A121" s="2" t="n"/>
       <c r="D121" s="5" t="n"/>
       <c r="E121" s="5" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="4" t="n"/>
+      <c r="A122" s="2" t="n"/>
       <c r="D122" s="5" t="n"/>
       <c r="E122" s="5" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="4" t="n"/>
+      <c r="A123" s="2" t="n"/>
       <c r="D123" s="5" t="n"/>
       <c r="E123" s="5" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="4" t="n"/>
+      <c r="A124" s="2" t="n"/>
       <c r="D124" s="5" t="n"/>
       <c r="E124" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:E124"/>
   <dataValidations count="3">
-    <dataValidation sqref="A5:A124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Date hors periode" error="Choisis une date dans la liste. Renseigne d'abord la date d'envoi dans la feuille Periode." type="list">
+    <dataValidation sqref="A5:A124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Date hors periode" error="Choisis une date dans la liste deroulante. Les dates proposees sont rappelees en haut de cette feuille." type="list">
       <formula1>=Periode!$B$7:$B$27</formula1>
     </dataValidation>
     <dataValidation sqref="B5:B124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Magasin inconnu" error="Choisis un magasin dans la liste déroulante." type="list">
@@ -1147,27 +1160,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>magasin</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>nom</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>code_postal</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>ville</t>
         </is>
@@ -6105,7 +6118,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>commercial</t>
         </is>
@@ -6164,7 +6177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6174,10 +6187,28 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Date d'envoi (le jeudi) :</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="n"/>
+          <t>Date de référence :</t>
+        </is>
+      </c>
+      <c r="B1" s="7">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="C1" s="8">
+        <f>$B$1</f>
+        <v/>
+      </c>
+      <c r="D1" s="6">
+        <f>IF(WEEKDAY($B$1,2)=4,"OK — bien un jeudi","⚠ PAS un jeudi — normal si tu remplis un autre jour")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Elle se met à jour toute seule. Ne la modifie que si tu remplis en retard.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6194,223 +6225,223 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>jour</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8">
+      <c r="A7" s="9">
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <f>$B$1</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8">
+      <c r="A8" s="9">
         <f>$B$1-1</f>
         <v/>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <f>$B$1-1</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8">
+      <c r="A9" s="9">
         <f>$B$1-2</f>
         <v/>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <f>$B$1-2</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8">
+      <c r="A10" s="9">
         <f>$B$1-3</f>
         <v/>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="2">
         <f>$B$1-3</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8">
+      <c r="A11" s="9">
         <f>$B$1-4</f>
         <v/>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="2">
         <f>$B$1-4</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8">
+      <c r="A12" s="9">
         <f>$B$1-5</f>
         <v/>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="2">
         <f>$B$1-5</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8">
+      <c r="A13" s="9">
         <f>$B$1-6</f>
         <v/>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="2">
         <f>$B$1-6</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8">
+      <c r="A14" s="9">
         <f>$B$1-7</f>
         <v/>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="2">
         <f>$B$1-7</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8">
+      <c r="A15" s="9">
         <f>$B$1-8</f>
         <v/>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="2">
         <f>$B$1-8</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8">
+      <c r="A16" s="9">
         <f>$B$1-9</f>
         <v/>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="2">
         <f>$B$1-9</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8">
+      <c r="A17" s="9">
         <f>$B$1-10</f>
         <v/>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <f>$B$1-10</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8">
+      <c r="A18" s="9">
         <f>$B$1-11</f>
         <v/>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <f>$B$1-11</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8">
+      <c r="A19" s="9">
         <f>$B$1-12</f>
         <v/>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <f>$B$1-12</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8">
+      <c r="A20" s="9">
         <f>$B$1-13</f>
         <v/>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <f>$B$1-13</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8">
+      <c r="A21" s="9">
         <f>$B$1-14</f>
         <v/>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="2">
         <f>$B$1-14</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8">
+      <c r="A22" s="9">
         <f>$B$1-15</f>
         <v/>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="2">
         <f>$B$1-15</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8">
+      <c r="A23" s="9">
         <f>$B$1-16</f>
         <v/>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="2">
         <f>$B$1-16</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8">
+      <c r="A24" s="9">
         <f>$B$1-17</f>
         <v/>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="2">
         <f>$B$1-17</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8">
+      <c r="A25" s="9">
         <f>$B$1-18</f>
         <v/>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="2">
         <f>$B$1-18</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8">
+      <c r="A26" s="9">
         <f>$B$1-19</f>
         <v/>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="2">
         <f>$B$1-19</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8">
+      <c r="A27" s="9">
         <f>$B$1-20</f>
         <v/>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="2">
         <f>$B$1-20</f>
         <v/>
       </c>
@@ -6426,14 +6457,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Comment remplir ce classeur</t>
         </is>
@@ -6442,14 +6473,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Feuille « Periode » : inscris la DATE D'ENVOI (le jeudi) dans la case bleutée.</t>
+          <t>1. Il n'y a AUCUNE date à taper. La feuille « Periode » se cale toute seule sur le jour</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Les 21 jours qui la précèdent se calculent tout seuls et alimentent la liste des dates.</t>
+          <t xml:space="preserve">   où tu ouvres le classeur, et propose les 21 jours qui précèdent.</t>
         </is>
       </c>
     </row>
@@ -6468,57 +6499,61 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   La période proposée est rappelée en haut de la feuille « Passages ».</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2. Feuille « Passages » : une ligne par passage effectué.</t>
+          <t xml:space="preserve">   (Si tu remplis longtemps après coup, tu peux forcer la date de référence en B1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   · date_visite  → choisis dans la liste (les 21 derniers jours)</t>
+          <t xml:space="preserve">   de la feuille « Periode » — le jour de la semaine s'affiche à côté pour te contrôler.)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   · magasin      → choisis dans la liste (les 182 points de vente)</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   · commercial   → choisis dans la liste</t>
+          <t>2. Feuille « Passages » : une ligne par passage effectué.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   · heures       → facultatives. Si tu les as, elles nous donnent la durée réelle des visites.</t>
+          <t xml:space="preserve">   · date_visite  → choisis dans la liste (les 21 derniers jours)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   · magasin      → choisis dans la liste (les 182 points de vente)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3. N'inscris QUE les passages réellement effectués. Une visite prévue mais non faite</t>
+          <t xml:space="preserve">   · commercial   → choisis dans la liste</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ne doit pas figurer : c'est ce qui a eu lieu qui nous intéresse.</t>
+          <t xml:space="preserve">   · heures       → facultatives. Si tu les as, elles nous donnent la durée réelle des visites.</t>
         </is>
       </c>
     </row>
@@ -6528,36 +6563,53 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4. Enregistre normalement (Ctrl+S) et envoie-nous LE CLASSEUR, tel quel.</t>
+          <t>3. N'inscris QUE les passages réellement effectués. Une visite prévue mais non faite</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pas de conversion, pas d'export CSV : notre application lit le .xlsx</t>
+          <t xml:space="preserve">   ne doit pas figurer : c'est ce qui a eu lieu qui nous intéresse.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   et va chercher la feuille « Passages » toute seule.</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>4. Enregistre normalement (Ctrl+S) et envoie-nous LE CLASSEUR, tel quel.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Le classeur se réutilise chaque semaine : il suffit de changer la date d'envoi</t>
+          <t xml:space="preserve">   Pas de conversion, pas d'export CSV : notre application lit le .xlsx</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   et va chercher la feuille « Passages » toute seule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Le classeur se réutilise chaque semaine : il suffit de changer la date d'envoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>et d'effacer les lignes précédentes.</t>
         </is>

</xml_diff>